<commit_message>
Fill whiteboard KPI dashboard with data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NLJUeWdK6NiYttMcUfGWXW
</commit_message>
<xml_diff>
--- a/KPI_Dashboard_Board.xlsx
+++ b/KPI_Dashboard_Board.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">Date: Friday, 23rd Oct 2026</t>
   </si>
@@ -46,24 +46,41 @@
     <t xml:space="preserve">Qualified Leads</t>
   </si>
   <si>
+    <t xml:space="preserve">CRM / Entry Forms</t>
+  </si>
+  <si>
     <t xml:space="preserve">No. of Paid Enrolments</t>
   </si>
   <si>
+    <t xml:space="preserve">Payment System</t>
+  </si>
+  <si>
     <t xml:space="preserve">Advertising Spend</t>
   </si>
   <si>
+    <t xml:space="preserve">Google &amp; Meta Ads Manager</t>
+  </si>
+  <si>
     <t xml:space="preserve">Revenue Generated</t>
   </si>
   <si>
+    <t xml:space="preserve">Accounting System</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gross Profit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit &amp; Loss Statement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -160,7 +177,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -181,7 +198,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -384,7 +409,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -418,61 +443,91 @@
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5" t="str">
+      <c r="B5" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>460</v>
+      </c>
+      <c r="D5" s="5" t="n">
         <f aca="false">IF(OR(B5="",C5=""),"",C5-B5)</f>
-        <v/>
-      </c>
-      <c r="E5" s="5"/>
+        <v>-40</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5" t="str">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>132</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <f aca="false">IF(OR(B6="",C6=""),"",C6-B6)</f>
-        <v/>
-      </c>
-      <c r="E6" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5" t="str">
+        <v>11</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>5940</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <f aca="false">IF(OR(B7="",C7=""),"",C7-B7)</f>
-        <v/>
-      </c>
-      <c r="E7" s="5"/>
+        <v>-60</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5" t="str">
+        <v>13</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>66000</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <f aca="false">IF(OR(B8="",C8=""),"",C8-B8)</f>
-        <v/>
-      </c>
-      <c r="E8" s="5"/>
+        <v>6000</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5" t="str">
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>22500</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <f aca="false">IF(OR(B9="",C9=""),"",C9-B9)</f>
-        <v/>
-      </c>
-      <c r="E9" s="5"/>
+        <v>-1500</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>